<commit_message>
chore(ag): adjust statistic complete date filter
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_ag/dossiers_service-afb.xlsx
+++ b/django/camac/statistics/config/kt_ag/dossiers_service-afb.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BED28D3-4ACF-4FFE-94F0-DB1B3160F049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B555FC-DF1E-44AE-9F37-529AA51DF187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="1620" windowWidth="20010" windowHeight="12885" tabRatio="887" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="33105" windowHeight="17610" tabRatio="887" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="21" r:id="rId8"/>
+    <pivotCache cacheId="23" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -83,9 +83,6 @@
     <t>&lt;= 30 Tage</t>
   </si>
   <si>
-    <t>31 - 60 Tage</t>
-  </si>
-  <si>
     <t>&gt; 60 Tage</t>
   </si>
   <si>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>Anzahl fristgerechte (60 Tage) erledigte Dossiers pro Zuständige Person</t>
+  </si>
+  <si>
+    <t>&lt;= 60 Tage</t>
   </si>
 </sst>
 </file>
@@ -436,8 +436,8 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="21">
     <cellStyle name="Accent" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -462,7 +462,13 @@
     <cellStyle name="Text" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
     <cellStyle name="Warning" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -483,7 +489,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46136.43192800926" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="20" xr:uid="{00000000-000A-0000-FFFF-FFFF50000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46146.443703240744" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="20" xr:uid="{00000000-000A-0000-FFFF-FFFF50000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:J1048576" sheet="Data"/>
   </cacheSource>
@@ -781,7 +787,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="PivotTable3" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" grandTotalCaption="Total Anzahl Dossiers" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="PivotTable3" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" grandTotalCaption="Total Anzahl Dossiers" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person">
   <location ref="A5:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" showAll="0"/>
@@ -827,7 +833,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000002000000}" name="PivotTable1" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0400-000002000000}" name="PivotTable1" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person">
   <location ref="A5:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -864,14 +870,14 @@
     <dataField name="Mittelwert von Durchlaufzeit in Tage" fld="6" subtotal="average" baseField="0" baseItem="0" numFmtId="1"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="1">
+    <format dxfId="3">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="2">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -891,7 +897,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B456AD4D-9646-4CC1-84EE-A09565AD0DDF}" name="PivotTable1" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist erreicht">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B456AD4D-9646-4CC1-84EE-A09565AD0DDF}" name="PivotTable1" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist erreicht">
   <location ref="G5:H8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" showAll="0"/>
@@ -950,7 +956,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0500-000003000000}" name="PivotTable2" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist erreicht">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0500-000003000000}" name="PivotTable2" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist erreicht">
   <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" showAll="0"/>
@@ -1009,7 +1015,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0600-000004000000}" name="PivotTable4" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Dossiertyp">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0600-000004000000}" name="PivotTable4" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Dossiertyp">
   <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" showAll="0"/>
@@ -1068,7 +1074,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0700-000005000000}" name="PivotTable5" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Gemeinde" colHeaderCaption="Dossiertyp">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0700-000005000000}" name="PivotTable5" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Gemeinde" colHeaderCaption="Dossiertyp">
   <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" showAll="0"/>
@@ -1554,10 +1560,10 @@
         <v>11</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1575,20 +1581,20 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIFS(Data!G:G,"&gt;30",Data!G:G,"&lt;=60")</f>
+        <f>COUNTIF(Data!G:G,"&lt;=60")</f>
         <v>0</v>
       </c>
       <c r="C7" s="16" t="e">
-        <f>COUNTIFS(Data!G:G,"&gt;30",Data!G:G,"&lt;=60") / B9</f>
+        <f>COUNTIF(Data!G:G,"&lt;=60") / B9</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="7">
         <f>COUNTIF(Data!G:G,"&gt;60")</f>
@@ -1601,10 +1607,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="8">
-        <f>SUM(B6:B8)</f>
+        <f>COUNTIF(Data!G:G,"&gt;=0")</f>
         <v>0</v>
       </c>
       <c r="C9" s="8"/>
@@ -1624,32 +1630,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75">
-      <c r="A1" s="20" t="s">
-        <v>23</v>
+      <c r="A1" s="19" t="s">
+        <v>22</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="19"/>
+        <v>16</v>
+      </c>
+      <c r="B6" s="20"/>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="19"/>
+        <v>21</v>
+      </c>
+      <c r="B7" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1666,30 +1672,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75">
-      <c r="A1" s="20" t="s">
-        <v>25</v>
+      <c r="A1" s="19" t="s">
+        <v>24</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="18"/>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="18"/>
     </row>
@@ -1725,52 +1731,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.75">
-      <c r="A1" s="20" t="s">
-        <v>33</v>
+      <c r="A1" s="19" t="s">
+        <v>32</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
+        <v>16</v>
+      </c>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
       <c r="G7" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H7" s="12" t="e">
         <v>#DIV/0!</v>
@@ -1778,12 +1784,12 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
+        <v>29</v>
+      </c>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
       <c r="G8" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H8" s="12" t="e">
         <v>#DIV/0!</v>
@@ -1811,50 +1817,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A1" s="20" t="s">
-        <v>28</v>
+      <c r="A1" s="19" t="s">
+        <v>27</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="H2" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
+        <v>16</v>
+      </c>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
+        <v>17</v>
+      </c>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1907,18 +1913,18 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1926,25 +1932,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
+        <v>16</v>
+      </c>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
+        <v>17</v>
+      </c>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>